<commit_message>
Support room-spanning and roomless dance-schedule sessions
Replace the single room field with a location union (located/roomless)
so a session can span multiple rooms or have no room at all (e.g. a
lunch break). Authors declare this in the spreadsheet with a ROOMS:
metadata line (mirroring the existing GCA: line) or a ditto mark for
the common contiguous-room case, since the parsing library has no
merged-cell support. Adds two real examples to the source spreadsheet
to exercise the new parsing end-to-end.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/dance-schedule.xlsx
+++ b/data/dance-schedule.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="183">
   <si>
     <t>Time</t>
   </si>
@@ -259,6 +259,9 @@
     <t>SSD : All Callers Dance - All Callers</t>
   </si>
   <si>
+    <t>"</t>
+  </si>
+  <si>
     <t>11:00a-12:00p</t>
   </si>
   <si>
@@ -437,6 +440,13 @@
     <t>SSD : Moonshine Tip - Dayle Hodge &amp; Karla Westphal</t>
   </si>
   <si>
+    <t>12:00p-1:30p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">* Lunch Break
+ROOMS: NONE</t>
+  </si>
+  <si>
     <t>9:00a-10:00a</t>
   </si>
   <si>
@@ -655,6 +665,9 @@
   </si>
   <si>
     <t>Plus : GCA Caller Showcase Dance - Karin Rabe &amp; Greg Moore</t>
+  </si>
+  <si>
+    <t>12:00p-2:00p</t>
   </si>
 </sst>
 </file>
@@ -729,7 +742,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -741,6 +754,12 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1303,7 +1322,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1346,7 +1365,9 @@
       <c r="B2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
@@ -1356,27 +1377,27 @@
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1384,26 +1405,26 @@
         <v>16</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1411,24 +1432,24 @@
         <v>24</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1436,26 +1457,26 @@
         <v>31</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1463,26 +1484,26 @@
         <v>39</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1490,24 +1511,24 @@
         <v>48</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1515,24 +1536,24 @@
         <v>55</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1542,13 +1563,21 @@
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
+    </row>
+    <row r="11" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>116</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1560,7 +1589,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1601,256 +1630,264 @@
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="4" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>21</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="J5" s="4"/>
     </row>
     <row r="6" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="I7" s="4"/>
       <c r="J7" s="4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="4" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="I10" s="4"/>
       <c r="J10" s="4" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
       <c r="F11" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="I11" s="4"/>
       <c r="J11" s="4" t="s">
-        <v>178</v>
+        <v>181</v>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>